<commit_message>
Abide in Me: light-is-life rule, emotional turns and living-water overflow
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UC78tJbpLPyZ6XAbTKxNP8
</commit_message>
<xml_diff>
--- a/abide-in-me/Abide-in-Me-Shot-Sheet.xlsx
+++ b/abide-in-me/Abide-in-Me-Shot-Sheet.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="597">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="599">
   <si>
     <t xml:space="preserve">Abide in Me — LTX shot sheet</t>
   </si>
@@ -33,6 +33,12 @@
     <t xml:space="preserve">Album: God Is About to Show Up, track 2 (reprise), 4:56 · Divine Ensemble · Production: Dazadi Music</t>
   </si>
   <si>
+    <t xml:space="preserve">THE RULE: The light is the life of God: His presence, Spirit, living water, Word and love. Wherever it works, two things must show: the physical signs of life (grey to warm, still to breathing, dry to green, cold to warm, a closed face opening, one becoming many) and, above all, a real emotional turn on a human face (delight, relief, being seen, forgiven or loved, reunion, laughter through tears). It behaves like living water: it wells up inside a person, pools in the chest, overflows out through the hands and tears, flows into the next person, and at the end the many springs become one river.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every shot is tested against it: where the light works, a real emotional turn must show on a face.</t>
+  </si>
+  <si>
     <t xml:space="preserve">One row per shot, 44 shots, one clip each, covering the whole song with no gaps and no repeats.</t>
   </si>
   <si>
@@ -117,22 +123,22 @@
     <t xml:space="preserve">A single point of light that opens into a glowing Hebrew letter aleph</t>
   </si>
   <si>
-    <t xml:space="preserve">One point of light breathes in the dark, slowly swelling and dimming like a heartbeat, then opens into a single glowing Hebrew letter, aleph, made of soft living fire.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A warm-gold darkness with no floor, no sky and no horizon, deep as the inside of a closed eye.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drifts forward through the dark toward the light, weightless, as if carried on breath. Ends on: The aleph glows alone and close in the center of the dark.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total darkness warmed to deep amber; one breathing point of gold light as the only source, grows from nothing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hush. Something is about to be spoken. Awe before beginning; the stillness before a voice.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Word (dream). A dreamlike, formless world: an endless warm-gold darkness like the inside of a dream, soft and illogical, where living Hebrew letters made of light drift, breathe and change shape. Sense: The faint warmth of a candle seen through closed eyelids; a low hum you feel more than hear.</t>
+    <t xml:space="preserve">A single drop of golden light falls from above into still dark water; slow rings spread across the surface, and from the center a single glowing Hebrew letter, aleph, rises out of the water made of soft living fire.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A warm-gold darkness with no floor, no sky and no horizon, only a surface of still dark water, deep as the inside of a closed eye.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drifts forward through the dark toward the light, weightless, as if carried on breath. Ends on: Close on the aleph glowing just above the rippling water.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total darkness warmed to deep amber; one falling drop of gold light as the only source, its glow spreading in rings across still water</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emotional turn: Hush, then a single drop: life about to begin. Hush. Something is about to be spoken. Awe before beginning; the stillness before a voice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Word (dream). A dreamlike, formless world: an endless warm-gold darkness like the inside of a dream, soft and illogical, where living Hebrew letters made of light drift, breathe and change shape. Sense: The plink of one drop in a silent room; a low hum you feel more than hear.</t>
   </si>
   <si>
     <t xml:space="preserve">No stars, planets or space imagery; no sudden flash; no readable caption; the light grows from nothing, never pops on. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
@@ -144,7 +150,7 @@
     <t xml:space="preserve">Text only: no faces to keep matching, and the loose invented look helps the dream</t>
   </si>
   <si>
-    <t xml:space="preserve">A dreamlike, formless world: an endless warm-gold darkness like the inside of a dream, soft and illogical, where living Hebrew letters made of light drift, breathe and change shape. A warm-gold darkness with no floor, no sky and no horizon, deep as the inside of a closed eye. One point of light breathes in the dark, slowly swelling and dimming like a heartbeat, then opens into a single glowing Hebrew letter, aleph, made of soft living fire. The camera drifts forward through the dark toward the light, weightless, as if carried on breath. The color stays warm gold, and any light grows slowly from nothing, never flashing. 50mm lens, soft focus at the edges. The shot ends: the aleph glows alone and close in the center of the dark.
+    <t xml:space="preserve">A dreamlike, formless world: an endless warm-gold darkness like the inside of a dream, soft and illogical, where living Hebrew letters made of light drift, breathe and change shape. A warm-gold darkness with no floor, no sky and no horizon, only a surface of still dark water, deep as the inside of a closed eye. A single drop of golden light falls from above into still dark water; slow rings spread across the surface, and from the center a single glowing Hebrew letter, aleph, rises out of the water made of soft living fire. The camera drifts forward through the dark toward the light, weightless, as if carried on breath. The color stays warm gold, and any light grows slowly from nothing, never flashing. 50mm lens, soft focus at the edges. The shot ends: close on the aleph glowing just above the rippling water.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -175,7 +181,7 @@
     <t xml:space="preserve">Dark gold ambience; each rising letter is its own soft light source, reflected in still dark water below</t>
   </si>
   <si>
-    <t xml:space="preserve">Wonder. The Word stirs. Like waking inside a dream and knowing it means something.</t>
+    <t xml:space="preserve">Emotional turn: Wonder as the Word stirs. Wonder. The Word stirs. Like waking inside a dream and knowing it means something.</t>
   </si>
   <si>
     <t xml:space="preserve">The Word (dream). A dreamlike, formless world: an endless warm-gold darkness like the inside of a dream, soft and illogical, where living Hebrew letters made of light drift, breathe and change shape. Sense: Embers rising on warm air; ripples spreading without a sound.</t>
@@ -215,7 +221,7 @@
     <t xml:space="preserve">Light comes from inside the vine itself: golden sap pulsing up the trunk, everything else falling to warm dark</t>
   </si>
   <si>
-    <t xml:space="preserve">Life taking shape. Order out of the formless. The first breath of creation; the Word becoming something that lives.</t>
+    <t xml:space="preserve">Emotional turn: Awe as the Word grows into a living vine. Life taking shape. Order out of the formless. The first breath of creation; the Word becoming something that lives.</t>
   </si>
   <si>
     <t xml:space="preserve">The Word (dream). A dreamlike, formless world: an endless warm-gold darkness like the inside of a dream, soft and illogical, where living Hebrew letters made of light drift, breathe and change shape. Sense: The slow creak of growing wood; warmth rising like sap.</t>
@@ -243,7 +249,7 @@
     <t xml:space="preserve">The vine of light, and faint grey outlines of people of every age drifting away from it</t>
   </si>
   <si>
-    <t xml:space="preserve">Faint grey outlines of human figures float loose in the dark like unfinished pencil sketches, many of them, of every age; cut off from the vine, their thin lines flicker and fade as they drift away.</t>
+    <t xml:space="preserve">Faint grey outlines of human figures float loose in the dark like unfinished pencil sketches, many of them, of every age; cut off from the vine, their lines dry and crack like a parched riverbed, and they drift away thirsty, reaching toward the glow they cannot reach.</t>
   </si>
   <si>
     <t xml:space="preserve">The edges of the dream-dark, away from the glowing vine.</t>
@@ -255,7 +261,7 @@
     <t xml:space="preserve">Bright gold vine on one side as key light; the drifting grey figures lit only by its fading spill, cold at the edges</t>
   </si>
   <si>
-    <t xml:space="preserve">Ache. Something is missing in them. Longing; people who are only an outline of themselves.</t>
+    <t xml:space="preserve">Emotional turn: Thirst: people dry and reaching, cut off. Thirst. Something is missing in them. Longing; people who are only an outline of themselves.</t>
   </si>
   <si>
     <t xml:space="preserve">The Word (dream). A dreamlike, formless world: an endless warm-gold darkness like the inside of a dream, soft and illogical, where living Hebrew letters made of light drift, breathe and change shape. Sense: Cold air at the edge of a warm room; a sound fading out.</t>
@@ -264,7 +270,7 @@
     <t xml:space="preserve">Not frightening or ghostly horror; no faces in pain; just faint, hollow and drifting. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">A dreamlike, formless world: an endless warm-gold darkness like the inside of a dream, soft and illogical, where living Hebrew letters made of light drift, breathe and change shape. The edges of the dream-dark, away from the glowing vine. Faint grey outlines of human figures float loose in the dark like unfinished pencil sketches, many of them, of every age; cut off from the vine, their thin lines flicker and fade as they drift away. The camera pulls slowly back from the vine to reveal the drifting grey figures between it and the dark. The color stays warm gold, and any light grows slowly from nothing, never flashing. 35mm lens. The shot ends: wide: the bright vine on one side, the faint grey figures scattered and drifting in the dark.
+    <t xml:space="preserve">A dreamlike, formless world: an endless warm-gold darkness like the inside of a dream, soft and illogical, where living Hebrew letters made of light drift, breathe and change shape. The edges of the dream-dark, away from the glowing vine. Faint grey outlines of human figures float loose in the dark like unfinished pencil sketches, many of them, of every age; cut off from the vine, their lines dry and crack like a parched riverbed, and they drift away thirsty, reaching toward the glow they cannot reach. The camera pulls slowly back from the vine to reveal the drifting grey figures between it and the dark. The color stays warm gold, and any light grows slowly from nothing, never flashing. 35mm lens. The shot ends: wide: the bright vine on one side, the faint grey figures scattered and drifting in the dark.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -292,7 +298,7 @@
     <t xml:space="preserve">Flat early-dawn wash on parchment, grey ink, the faintest gold on the paper's edges</t>
   </si>
   <si>
-    <t xml:space="preserve">Recognition. This is our world, sketched. Ordinary life before it is alive.</t>
+    <t xml:space="preserve">Emotional turn: Ordinary life before it is alive. Recognition. This is our world, sketched. Ordinary life before it is alive.</t>
   </si>
   <si>
     <t xml:space="preserve">Drawn (2D). Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Sense: The scratch of a pen on paper; the hush of a city at dawn.</t>
@@ -323,19 +329,19 @@
     <t xml:space="preserve">Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan</t>
   </si>
   <si>
-    <t xml:space="preserve">A thin stream of tiny glowing Hebrew letters flows down from above like falling seeds and enters Ana's forehead; watercolor color floods her figure from the inside out, her yellow cardigan blooming, her face lighting up; she looks up and laughs.</t>
+    <t xml:space="preserve">A thin stream of tiny glowing Hebrew letters flows down like falling water and pools inside Ana's chest; watercolor color wells up through her from the inside out, her yellow cardigan blooming; she gasps, then bursts into delighted laughter, spinning with her arms open as the light spills off her fingertips.</t>
   </si>
   <si>
     <t xml:space="preserve">The drawn street at the building's front steps.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pushes slowly in on Ana as the color fills her. Ends on: Close on Ana's colored, laughing face amid the grey street.</t>
+    <t xml:space="preserve">Pushes slowly in on Ana as the color fills her. Ends on: Close on Ana laughing with pure joy, light dripping from her fingertips.</t>
   </si>
   <si>
     <t xml:space="preserve">Soft top light from the falling letters; watercolor color blooming warm from inside Ana</t>
   </si>
   <si>
-    <t xml:space="preserve">Delight. The first branch takes life. Joy as simple as a child's.</t>
+    <t xml:space="preserve">Emotional turn: Ana gasps, then bursts into laughter. Delight. The first branch takes life. Joy as simple as a child's.</t>
   </si>
   <si>
     <t xml:space="preserve">Drawn (2D). Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Sense: Warm water spreading through paper; a small bright laugh.</t>
@@ -344,7 +350,7 @@
     <t xml:space="preserve">The letters never land as a caption or readable line; no flash; color soaks in slowly like watercolor. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan. The drawn street at the building's front steps. A thin stream of tiny glowing Hebrew letters flows down from above like falling seeds and enters Ana's forehead; watercolor color floods her figure from the inside out, her yellow cardigan blooming, her face lighting up; she looks up and laughs. The camera pushes slowly in on Ana as the color fills her. The color stays warm gold, and any light grows slowly from nothing, never flashing. Close 2D framing. The shot ends: close on Ana's colored, laughing face amid the grey street.
+    <t xml:space="preserve">Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan. The drawn street at the building's front steps. A thin stream of tiny glowing Hebrew letters flows down like falling water and pools inside Ana's chest; watercolor color wells up through her from the inside out, her yellow cardigan blooming; she gasps, then bursts into delighted laughter, spinning with her arms open as the light spills off her fingertips. The camera pushes slowly in on Ana as the color fills her. The color stays warm gold, and any light grows slowly from nothing, never flashing. Close 2D framing. The shot ends: close on Ana laughing with pure joy, light dripping from her fingertips.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -360,19 +366,19 @@
     <t xml:space="preserve">Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan; Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves</t>
   </si>
   <si>
-    <t xml:space="preserve">Ana runs to her mother and takes her hand; color flows from the child's hand through their joined fingers up Rosa's arm until the tired grey woman blooms into warm color and kneels to hug her daughter.</t>
+    <t xml:space="preserve">Ana runs to her mother and grabs her hand; the light overflowing from the child pours like warm water through their joined fingers and up Rosa's tired grey arm; Rosa's face, numb with exhaustion, crumples into tears and a smile, and she drops to hug her daughter tight.</t>
   </si>
   <si>
     <t xml:space="preserve">The building's doorway at dawn; Rosa, still grey, coming home from her night shift.</t>
   </si>
   <si>
-    <t xml:space="preserve">Follows the flow of color along their joined arms, moving right to left. Ends on: Medium on mother and daughter embracing in full color in the grey doorway.</t>
+    <t xml:space="preserve">Follows the flow of color along their joined arms, moving right to left. Ends on: Medium on mother and daughter holding each other, Rosa crying and smiling, both in full color in the grey doorway.</t>
   </si>
   <si>
     <t xml:space="preserve">Dawn backlight in the doorway; warm color traveling up Rosa's arm as the brightest point</t>
   </si>
   <si>
-    <t xml:space="preserve">Tenderness. The light passes on. Love moving from one person to the next.</t>
+    <t xml:space="preserve">Emotional turn: Rosa's numb face crumples into tears and a smile. Relief. A tired mother is filled. Love moving from one person to the next.</t>
   </si>
   <si>
     <t xml:space="preserve">Drawn (2D). Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Sense: A small warm hand in a cold one.</t>
@@ -381,7 +387,7 @@
     <t xml:space="preserve">Rosa is not made to kneel in worship, only to hug her daughter; no sparkles, the color flows like ink. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. The building's doorway at dawn; Rosa, still grey, coming home from her night shift. Ana runs to her mother and takes her hand; color flows from the child's hand through their joined fingers up Rosa's arm until the tired grey woman blooms into warm color and kneels to hug her daughter. The camera follows the flow of color along their joined arms, moving right to left. The color stays warm gold, and any light grows slowly from nothing, never flashing. Medium 2D framing. The shot ends: medium on mother and daughter embracing in full color in the grey doorway.
+    <t xml:space="preserve">Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. The building's doorway at dawn; Rosa, still grey, coming home from her night shift. Ana runs to her mother and grabs her hand; the light overflowing from the child pours like warm water through their joined fingers and up Rosa's tired grey arm; Rosa's face, numb with exhaustion, crumples into tears and a smile, and she drops to hug her daughter tight. The camera follows the flow of color along their joined arms, moving right to left. The color stays warm gold, and any light grows slowly from nothing, never flashing. Medium 2D framing. The shot ends: medium on mother and daughter holding each other, Rosa crying and smiling, both in full color in the grey doorway.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -409,7 +415,7 @@
     <t xml:space="preserve">Light stream glowing warm at the alley mouth behind camera; David walks into flat grey shade</t>
   </si>
   <si>
-    <t xml:space="preserve">Sorrow. A branch refuses. The ache of watching someone you love choose the dark.</t>
+    <t xml:space="preserve">Emotional turn: Sorrow as David turns away. Sorrow. A branch refuses. The ache of watching someone you love choose the dark.</t>
   </si>
   <si>
     <t xml:space="preserve">Drawn (2D). Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Sense: Footsteps fading; a door closing somewhere.</t>
@@ -446,7 +452,7 @@
     <t xml:space="preserve">Warm gold-leaf sunlight across the drawn vineyard; Yeshua's outline is the brightest light in frame</t>
   </si>
   <si>
-    <t xml:space="preserve">Gentle authority. He is the source. Peace; the one everything flows from.</t>
+    <t xml:space="preserve">Emotional turn: Peace in the presence of the source. Gentle authority. He is the source. Peace; the one everything flows from.</t>
   </si>
   <si>
     <t xml:space="preserve">Drawn (2D). Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Sense: Sun-warmed leaves; a calm voice you don't hear but feel.</t>
@@ -471,19 +477,19 @@
     <t xml:space="preserve">Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat</t>
   </si>
   <si>
-    <t xml:space="preserve">Tiny glowing Hebrew letters drift into his head like seeds into soil; inside his drawn outline they spread into a constellation of light through his mind, then run down like roots into his chest, and his heart glows; he lifts his eyes, color rising through him.</t>
+    <t xml:space="preserve">Tiny glowing Hebrew letters drift into his head like seeds into soil, spread into a constellation through his mind, then run down like water into his chest and pool there, rising; his tired face goes still, his eyes fill with tears, and a slow, disbelieving smile breaks across it as color floods through him.</t>
   </si>
   <si>
     <t xml:space="preserve">Close on Tomas on the drawn building site, hard hat in hand, tired.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pushes in slowly toward his head, then tilts down to his chest following the light. Ends on: Close on Tomas's face lifting, the glow in his chest.</t>
+    <t xml:space="preserve">Pushes in slowly toward his head, then tilts down to his chest following the light. Ends on: Close on Tomas's wet eyes and breaking smile, light welling in his chest.</t>
   </si>
   <si>
     <t xml:space="preserve">Muted grey site light; a constellation of gold inside his head and chest becomes the key light</t>
   </si>
   <si>
-    <t xml:space="preserve">Revelation. Understanding dawns. The moment knowledge becomes life.</t>
+    <t xml:space="preserve">Emotional turn: Tomas's eyes fill; a disbelieving smile. Being seen. Understanding becomes joy. The moment knowledge becomes life.</t>
   </si>
   <si>
     <t xml:space="preserve">Drawn (2D). Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Sense: Like a thought arriving in perfect silence.</t>
@@ -492,7 +498,7 @@
     <t xml:space="preserve">Not a sci-fi brain scan or circuitry; letters stay soft and gold; no flash. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. Close on Tomas on the drawn building site, hard hat in hand, tired. Tiny glowing Hebrew letters drift into his head like seeds into soil; inside his drawn outline they spread into a constellation of light through his mind, then run down like roots into his chest, and his heart glows; he lifts his eyes, color rising through him. The camera pushes in slowly toward his head, then tilts down to his chest following the light. The color stays warm gold, and any light grows slowly from nothing, never flashing. Close 2D framing. The shot ends: close on Tomas's face lifting, the glow in his chest.
+    <t xml:space="preserve">Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. Close on Tomas on the drawn building site, hard hat in hand, tired. Tiny glowing Hebrew letters drift into his head like seeds into soil, spread into a constellation through his mind, then run down like water into his chest and pool there, rising; his tired face goes still, his eyes fill with tears, and a slow, disbelieving smile breaks across it as color floods through him. The camera pushes in slowly toward his head, then tilts down to his chest following the light. The color stays warm gold, and any light grows slowly from nothing, never flashing. Close 2D framing. The shot ends: close on Tomas's wet eyes and breaking smile, light welling in his chest.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -508,7 +514,7 @@
     <t xml:space="preserve">Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan; Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves; Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat; Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds; Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane</t>
   </si>
   <si>
-    <t xml:space="preserve">A thread of light like a vine runs through the walls from apartment to apartment, linking each person; Rosa, Tomas and Ana glow in color, Eli and Samuel still grey but the vine of light reaching toward them.</t>
+    <t xml:space="preserve">Light flows like a stream of living water through the walls from apartment to apartment, linking each person; in their kitchen Rosa and Ana laugh together, Tomas on the stairs pauses and smiles at the warmth, while upstairs Eli and Samuel are still grey and the stream is reaching toward their doors.</t>
   </si>
   <si>
     <t xml:space="preserve">The whole drawn apartment building seen like an open dollhouse: Ana and Rosa in their kitchen, Tomas on the stairs, Eli in his room, Samuel alone upstairs.</t>
@@ -520,7 +526,7 @@
     <t xml:space="preserve">Night interior washes in each room; the vine of light through the walls is the main source, brighter where people are lit</t>
   </si>
   <si>
-    <t xml:space="preserve">Belonging. Many become one. One body; nobody is separate.</t>
+    <t xml:space="preserve">Emotional turn: A home laughing together as the light flows. Belonging. Many become one. One body; nobody is separate.</t>
   </si>
   <si>
     <t xml:space="preserve">Drawn (2D). Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Sense: The building creaking and breathing together like one house.</t>
@@ -529,7 +535,7 @@
     <t xml:space="preserve">No floor-plan diagram look; no captions or names on doors; keep it hand-drawn and warm. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. The whole drawn apartment building seen like an open dollhouse: Ana and Rosa in their kitchen, Tomas on the stairs, Eli in his room, Samuel alone upstairs. A thread of light like a vine runs through the walls from apartment to apartment, linking each person; Rosa, Tomas and Ana glow in color, Eli and Samuel still grey but the vine of light reaching toward them. The camera flows in one unbroken move up through the building from floor to floor. The color stays warm gold, and any light grows slowly from nothing, never flashing. Wide 2D framing. The shot ends: wide on the whole building, the vine of light running through it.
+    <t xml:space="preserve">Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. The whole drawn apartment building seen like an open dollhouse: Ana and Rosa in their kitchen, Tomas on the stairs, Eli in his room, Samuel alone upstairs. Light flows like a stream of living water through the walls from apartment to apartment, linking each person; in their kitchen Rosa and Ana laugh together, Tomas on the stairs pauses and smiles at the warmth, while upstairs Eli and Samuel are still grey and the stream is reaching toward their doors. The camera flows in one unbroken move up through the building from floor to floor. The color stays warm gold, and any light grows slowly from nothing, never flashing. Wide 2D framing. The shot ends: wide on the whole building, the vine of light running through it.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -560,7 +566,7 @@
     <t xml:space="preserve">Pale, cool, shadowless daylight; no gold, only a little warmth on the drifting dust</t>
   </si>
   <si>
-    <t xml:space="preserve">Gravity. Without Him, nothing lasts. Sober truth, not fear.</t>
+    <t xml:space="preserve">Emotional turn: The sober stillness of dry branches. Gravity. Without Him, nothing lasts. Sober truth, not fear.</t>
   </si>
   <si>
     <t xml:space="preserve">Drawn (2D). Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Sense: Dry leaves skittering; wind across a field.</t>
@@ -597,7 +603,7 @@
     <t xml:space="preserve">Cold white sparkle of drawn coins and signs against charcoal dark; no warmth anywhere</t>
   </si>
   <si>
-    <t xml:space="preserve">Grief. The lost one goes further. Losing someone to the world.</t>
+    <t xml:space="preserve">Emotional turn: Grief as David is carried off. Grief. The lost one goes further. Losing someone to the world.</t>
   </si>
   <si>
     <t xml:space="preserve">Drawn (2D). Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Sense: A thread snapping; wind rising.</t>
@@ -625,19 +631,19 @@
     <t xml:space="preserve">Yeshua as a tall figure outlined in gold light, cream tunic and striped mantle, no drawn face; Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat</t>
   </si>
   <si>
-    <t xml:space="preserve">Yeshua's hand of light trims the branch with a small knife; beside it, Tomas lets go of a fat envelope of shortcut money he was offered, and it falls away; where the cut was made, new green shoots bud at once.</t>
+    <t xml:space="preserve">Yeshua's hand of light trims the fruitless branch with a small knife; beside it Tomas, gripping a fat envelope of shortcut money, hesitates, then lets it fall; his shoulders drop as if a weight has gone, he exhales and laughs with relief, and where the cut was made new green shoots bud at once.</t>
   </si>
   <si>
     <t xml:space="preserve">The drawn vineyard again, a lit branch heavy with leaves but no fruit.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pushes in slowly on the cut, then eases down to the new shoots. Ends on: Close on the fresh green shoots budding from the cut branch.</t>
+    <t xml:space="preserve">Pushes in slowly on the cut, then eases down to the new shoots. Ends on: Close on the fresh green shoots, Tomas's relieved face soft behind them.</t>
   </si>
   <si>
     <t xml:space="preserve">Soft morning gold on the vineyard; a small bright spot where the cut is made, fresh green catching the light</t>
   </si>
   <si>
-    <t xml:space="preserve">A clean, hard mercy. Pruning hurts, and it is love.</t>
+    <t xml:space="preserve">Emotional turn: Tomas lets go, exhales and laughs with relief. A clean, hard mercy, and the relief after it. Pruning hurts, and it is love.</t>
   </si>
   <si>
     <t xml:space="preserve">Drawn (2D). Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Sense: A clean snip; sap beading at the cut.</t>
@@ -646,7 +652,7 @@
     <t xml:space="preserve">No blood, no harsh cutting of people; the knife only touches the vine. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Yeshua is drawn as a tall figure outlined in living gold light, in a cream tunic and a striped mantle, his face a soft glow with no drawn features. He never sings or mouths words. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. The drawn vineyard again, a lit branch heavy with leaves but no fruit. Yeshua's hand of light trims the branch with a small knife; beside it, Tomas lets go of a fat envelope of shortcut money he was offered, and it falls away; where the cut was made, new green shoots bud at once. The camera pushes in slowly on the cut, then eases down to the new shoots. The color stays warm gold, and any light grows slowly from nothing, never flashing. Close 2D framing. The shot ends: close on the fresh green shoots budding from the cut branch.
+    <t xml:space="preserve">Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Yeshua is drawn as a tall figure outlined in living gold light, in a cream tunic and a striped mantle, his face a soft glow with no drawn features. He never sings or mouths words. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. The drawn vineyard again, a lit branch heavy with leaves but no fruit. Yeshua's hand of light trims the fruitless branch with a small knife; beside it Tomas, gripping a fat envelope of shortcut money, hesitates, then lets it fall; his shoulders drop as if a weight has gone, he exhales and laughs with relief, and where the cut was made new green shoots bud at once. The camera pushes in slowly on the cut, then eases down to the new shoots. The color stays warm gold, and any light grows slowly from nothing, never flashing. Close 2D framing. The shot ends: close on the fresh green shoots, Tomas's relieved face soft behind them.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -674,7 +680,7 @@
     <t xml:space="preserve">Late golden sun rising through the vineyard; warm rim light on the children, the page edges catching depth shadows</t>
   </si>
   <si>
-    <t xml:space="preserve">Gladness. The fruit is people. Life multiplying; a future.</t>
+    <t xml:space="preserve">Emotional turn: Children's joy, the fruit running free. Gladness. The fruit is people. Life multiplying; a future.</t>
   </si>
   <si>
     <t xml:space="preserve">Drawn (2D). Hand-drawn 2D animation in fine ink line and gold-leaf watercolor on warm parchment, like an illuminated manuscript that has come alive; flat, with no real depth yet. Sense: Children's feet on stone; paper rustling as it lifts.</t>
@@ -708,7 +714,7 @@
     <t xml:space="preserve">Golden afternoon sun raking low, creating the first real shadows as the street rises into 3D</t>
   </si>
   <si>
-    <t xml:space="preserve">Rising strength. The world gets weight. The music swells; something serious is beginning.</t>
+    <t xml:space="preserve">Emotional turn: The swell: the world gains weight. Rising strength. The world gets weight. The music swells; something serious is beginning.</t>
   </si>
   <si>
     <t xml:space="preserve">Sculpted (3D). Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Sense: Paper turning to wood and stone; the hum growing louder.</t>
@@ -745,7 +751,7 @@
     <t xml:space="preserve">Huge cool moon as backlight; Yeshua a steady warm glow; the mirages a cold glittering gold that dies out</t>
   </si>
   <si>
-    <t xml:space="preserve">Determination. He chooses before He asks us to. Resolve; the hard choice made first by Him.</t>
+    <t xml:space="preserve">Emotional turn: Resolve: He refuses the world first. Determination. He chooses before He asks us to. Resolve; the hard choice made first by Him.</t>
   </si>
   <si>
     <t xml:space="preserve">Sculpted (3D). Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Sense: Desert wind; sand hissing over rock.</t>
@@ -770,19 +776,19 @@
     <t xml:space="preserve">Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds</t>
   </si>
   <si>
-    <t xml:space="preserve">Eli mouths along to someone else's song for his followers, performing a smile that isn't his; tiny glowing Hebrew letters drift through his window and into his mind; he stops, lowers the phone, and switches off the ring light.</t>
+    <t xml:space="preserve">Eli mouths along to someone else's song for his followers, performing a smile that isn't his; tiny glowing Hebrew letters drift through his window and pool inside him; he stops, lowers the phone and switches off the ring light, and in the quiet dark his real face appears: he breathes, his eyes fill, and a small, true smile comes.</t>
   </si>
   <si>
     <t xml:space="preserve">Eli's 3D bedroom at night, a ring light and his phone on a stand, a screen full of floating hearts and numbers.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pushes slowly in on his face as the cold ring light goes out and warm light rises in him. Ends on: Close on Eli's face in the dark room, warm light starting within him.</t>
+    <t xml:space="preserve">Pushes slowly in on his face as the cold ring light goes out and warm light rises in him. Ends on: Close on Eli's real smile and wet eyes in the dark room, warm light welling within him.</t>
   </si>
   <si>
     <t xml:space="preserve">Cold ring-light and phone glow on his face that switch off; warm light then rising softly from within him</t>
   </si>
   <si>
-    <t xml:space="preserve">The hard choice, mirrored. Choosing the real over the performance.</t>
+    <t xml:space="preserve">Emotional turn: Eli's real face, wet eyes, a true smile. The hard choice, mirrored. Choosing the real over the performance.</t>
   </si>
   <si>
     <t xml:space="preserve">Sculpted (3D). Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Sense: A notification chime cut short; quiet.</t>
@@ -791,7 +797,7 @@
     <t xml:space="preserve">Eli lip-syncs only a generic pop song with his mouth, never the lyrics of this song; no pink ring light; no brand logos. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. Eli's 3D bedroom at night, a ring light and his phone on a stand, a screen full of floating hearts and numbers. Eli mouths along to someone else's song for his followers, performing a smile that isn't his; tiny glowing Hebrew letters drift through his window and into his mind; he stops, lowers the phone, and switches off the ring light. The camera pushes slowly in on his face as the cold ring light goes out and warm light rises in him. The color stays warm gold, and any light grows slowly from nothing, never flashing. 85mm lens, shallow depth of field. The shot ends: close on Eli's face in the dark room, warm light starting within him.
+    <t xml:space="preserve">Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. Eli's 3D bedroom at night, a ring light and his phone on a stand, a screen full of floating hearts and numbers. Eli mouths along to someone else's song for his followers, performing a smile that isn't his; tiny glowing Hebrew letters drift through his window and pool inside him; he stops, lowers the phone and switches off the ring light, and in the quiet dark his real face appears: he breathes, his eyes fill, and a small, true smile comes. The camera pushes slowly in on his face as the cold ring light goes out and warm light rises in him. The color stays warm gold, and any light grows slowly from nothing, never flashing. 85mm lens, shallow depth of field. The shot ends: close on Eli's real smile and wet eyes in the dark room, warm light welling within him.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -819,7 +825,7 @@
     <t xml:space="preserve">Strong low sun ahead of them through moving cloud; long shadows behind, warm rim light on everyone</t>
   </si>
   <si>
-    <t xml:space="preserve">Set face; shared resolve. We follow because He went first.</t>
+    <t xml:space="preserve">Emotional turn: Shared resolve leaning into the wind. Set face; shared resolve. We follow because He went first.</t>
   </si>
   <si>
     <t xml:space="preserve">Sculpted (3D). Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Sense: Wind roaring; footsteps steady on stone.</t>
@@ -856,7 +862,7 @@
     <t xml:space="preserve">Cold gold-white glare from towers, screens and chandeliers; hard, dazzling, no warmth on David's face</t>
   </si>
   <si>
-    <t xml:space="preserve">Temptation; the pull of more. The ache of wanting what never satisfies.</t>
+    <t xml:space="preserve">Emotional turn: Hunger for what never satisfies. Temptation; the pull of more. The ache of wanting what never satisfies.</t>
   </si>
   <si>
     <t xml:space="preserve">Sculpted (3D). Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Sense: Glass chimes; a crowd's empty applause.</t>
@@ -893,7 +899,7 @@
     <t xml:space="preserve">Flat grey light as the glitter dies; dust in the air, no sun, colorless</t>
   </si>
   <si>
-    <t xml:space="preserve">Brokenness; the bottom of the lie. Emptiness after the world has taken everything.</t>
+    <t xml:space="preserve">Emotional turn: Emptiness at the bottom of the lie. Brokenness; the bottom of the lie. Emptiness after the world has taken everything.</t>
   </si>
   <si>
     <t xml:space="preserve">Sculpted (3D). Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Sense: Glass falling like dry rain; silence after.</t>
@@ -933,7 +939,7 @@
     <t xml:space="preserve">The same grey scene with one warm pool of light falling from the mantle onto David's shoulders</t>
   </si>
   <si>
-    <t xml:space="preserve">Mercy that waits. Love that has not given up on him.</t>
+    <t xml:space="preserve">Emotional turn: Mercy waiting, not yet received. Mercy that waits. Love that has not given up on him.</t>
   </si>
   <si>
     <t xml:space="preserve">Sculpted (3D). Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Sense: Rain stopping; warmth on the back of the neck.</t>
@@ -958,19 +964,19 @@
     <t xml:space="preserve">Rain of the Word</t>
   </si>
   <si>
-    <t xml:space="preserve">A soft rain of tiny glowing Hebrew letters begins to fall; where it lands, the dust darkens, a dry vine on the fence turns green, and Tomas straightens, the weight suddenly lighter, light glowing in his chest.</t>
+    <t xml:space="preserve">A soft rain of tiny glowing Hebrew letters begins to fall like living water; where it lands the dust darkens and a dry vine on the fence turns green; Tomas sets down the steel beam, lifts his face and open hands into the rain, and laughs out loud like a boy, tears and rain running together.</t>
   </si>
   <si>
     <t xml:space="preserve">A sculpted 3D building site in a dry, dusty heat; Tomas carrying a heavy steel beam.</t>
   </si>
   <si>
-    <t xml:space="preserve">Tilts up from the greening vine to Tomas's face lifted into the rain. Ends on: Medium on Tomas standing tall in the soft golden rain.</t>
+    <t xml:space="preserve">Tilts up from the greening vine to Tomas's face lifted into the rain. Ends on: Medium on Tomas laughing with his face and hands lifted into the golden rain.</t>
   </si>
   <si>
     <t xml:space="preserve">Hot hazy midday light, then soft gold as the rain of letters falls; the vine greening in the light</t>
   </si>
   <si>
-    <t xml:space="preserve">Relief. Refreshment after drought. Being refreshed from within.</t>
+    <t xml:space="preserve">Emotional turn: Tomas laughs like a boy in the rain. Relief. Refreshment after drought. Being refreshed from within.</t>
   </si>
   <si>
     <t xml:space="preserve">Sculpted (3D). Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Sense: First drops on hot dust; a long breath out.</t>
@@ -979,7 +985,7 @@
     <t xml:space="preserve">Letters fall softly like rain, never as readable text; no flash; no thunderstorm. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. A sculpted 3D building site in a dry, dusty heat; Tomas carrying a heavy steel beam. A soft rain of tiny glowing Hebrew letters begins to fall; where it lands, the dust darkens, a dry vine on the fence turns green, and Tomas straightens, the weight suddenly lighter, light glowing in his chest. The camera tilts up from the greening vine to Tomas's face lifted into the rain. The color stays warm gold, and any light grows slowly from nothing, never flashing. 50mm lens. The shot ends: medium on Tomas standing tall in the soft golden rain.
+    <t xml:space="preserve">Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. A sculpted 3D building site in a dry, dusty heat; Tomas carrying a heavy steel beam. A soft rain of tiny glowing Hebrew letters begins to fall like living water; where it lands the dust darkens and a dry vine on the fence turns green; Tomas sets down the steel beam, lifts his face and open hands into the rain, and laughs out loud like a boy, tears and rain running together. The camera tilts up from the greening vine to Tomas's face lifted into the rain. The color stays warm gold, and any light grows slowly from nothing, never flashing. 50mm lens. The shot ends: medium on Tomas laughing with his face and hands lifted into the golden rain.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -998,19 +1004,19 @@
     <t xml:space="preserve">Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves; Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds; Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat; Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan; Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane</t>
   </si>
   <si>
-    <t xml:space="preserve">In one room Rosa scrubs a floor after her shift; on the stairs Eli carries Samuel's groceries up five flights; in the kitchen Tomas cooks for Ana; through every wall a vine of light pulses brighter with each act.</t>
+    <t xml:space="preserve">In one room Rosa scrubs a floor after her shift; on the stairs Eli carries Samuel's groceries up five flights, and when Samuel opens his door the old man's face lights up in surprised delight; in the kitchen Tomas cooks for Ana; through every wall a stream of light flows like water, brighter with each act.</t>
   </si>
   <si>
     <t xml:space="preserve">The 3D apartment building opened like a dollhouse at night.</t>
   </si>
   <si>
-    <t xml:space="preserve">Flows in one unbroken move up through the building, room to room. Ends on: Wide on the whole building, the vine of light glowing through it.</t>
+    <t xml:space="preserve">Flows in one unbroken move up through the building, room to room. Ends on: Wide on the whole building, the stream of light glowing through it, Samuel smiling in his doorway.</t>
   </si>
   <si>
     <t xml:space="preserve">Night: a warm practical lamp in each room, the vine of light in the walls pulsing as a moving source</t>
   </si>
   <si>
-    <t xml:space="preserve">Persevering love; the hard chores done for others. Unseen faithfulness is the vine bearing fruit.</t>
+    <t xml:space="preserve">Emotional turn: Samuel's surprised delight at his door. Persevering love; the hard chores done for others. Unseen faithfulness is the vine bearing fruit.</t>
   </si>
   <si>
     <t xml:space="preserve">Sculpted (3D). Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Sense: A scrubbing brush, footsteps on stairs, a pan sizzling, all one rhythm.</t>
@@ -1019,7 +1025,7 @@
     <t xml:space="preserve">No split-screen or grid; one continuous move; nobody glows like a superhero. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. The 3D apartment building opened like a dollhouse at night. In one room Rosa scrubs a floor after her shift; on the stairs Eli carries Samuel's groceries up five flights; in the kitchen Tomas cooks for Ana; through every wall a vine of light pulses brighter with each act. The camera flows in one unbroken move up through the building, room to room. The color stays warm gold, and any light grows slowly from nothing, never flashing. 24mm lens, deep focus. The shot ends: wide on the whole building, the vine of light glowing through it.
+    <t xml:space="preserve">Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. The 3D apartment building opened like a dollhouse at night. In one room Rosa scrubs a floor after her shift; on the stairs Eli carries Samuel's groceries up five flights, and when Samuel opens his door the old man's face lights up in surprised delight; in the kitchen Tomas cooks for Ana; through every wall a stream of light flows like water, brighter with each act. The camera flows in one unbroken move up through the building, room to room. The color stays warm gold, and any light grows slowly from nothing, never flashing. 24mm lens, deep focus. The shot ends: wide on the whole building, the stream of light glowing through it, Samuel smiling in his doorway.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -1035,7 +1041,7 @@
     <t xml:space="preserve">Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves</t>
   </si>
   <si>
-    <t xml:space="preserve">Rosa pauses, closes her eyes, and a quiet constellation of glowing Hebrew letters turns inside her mind; she opens her eyes, nods as if she heard a voice, takes a bowl of soup and goes out the door toward the stairs to Samuel's.</t>
+    <t xml:space="preserve">Rosa pauses, closes her eyes, and a quiet constellation of glowing Hebrew letters turns inside her mind; her face softens with tender compassion and her eyes glisten; she nods as if she heard a voice, takes a bowl of soup and goes out the door toward the stairs to Samuel's.</t>
   </si>
   <si>
     <t xml:space="preserve">Rosa's small 3D kitchen at night, a mop leaning on the wall.</t>
@@ -1047,7 +1053,7 @@
     <t xml:space="preserve">Single warm kitchen bulb, dim; a small gold constellation glowing inside her mind on closed eyes</t>
   </si>
   <si>
-    <t xml:space="preserve">Listening. The Spirit speaks. Being led from within, then obeying.</t>
+    <t xml:space="preserve">Emotional turn: Rosa's tender compassion, eyes glistening. Listening. The Spirit speaks. Being led from within, then obeying.</t>
   </si>
   <si>
     <t xml:space="preserve">Sculpted (3D). Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Sense: A clock ticking; a whisper you can't quite hear.</t>
@@ -1056,7 +1062,7 @@
     <t xml:space="preserve">No literal voice bubble or text; not a vision of angels; the prompting is quiet and inward. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Rosa's small 3D kitchen at night, a mop leaning on the wall. Rosa pauses, closes her eyes, and a quiet constellation of glowing Hebrew letters turns inside her mind; she opens her eyes, nods as if she heard a voice, takes a bowl of soup and goes out the door toward the stairs to Samuel's. The camera pushes in slowly on her closed eyes, then follows her to the door. The color stays warm gold, and any light grows slowly from nothing, never flashing. 50mm lens. The shot ends: medium on Rosa at the door with the soup, looking up toward the stairs.
+    <t xml:space="preserve">Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Rosa's small 3D kitchen at night, a mop leaning on the wall. Rosa pauses, closes her eyes, and a quiet constellation of glowing Hebrew letters turns inside her mind; her face softens with tender compassion and her eyes glisten; she nods as if she heard a voice, takes a bowl of soup and goes out the door toward the stairs to Samuel's. The camera pushes in slowly on her closed eyes, then follows her to the door. The color stays warm gold, and any light grows slowly from nothing, never flashing. 50mm lens. The shot ends: medium on Rosa at the door with the soup, looking up toward the stairs.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -1081,7 +1087,7 @@
     <t xml:space="preserve">Warm stairwell bulb from above; light deepening on real skin as texture appears</t>
   </si>
   <si>
-    <t xml:space="preserve">Holy awe. It becomes real. The Word became flesh and dwelt among us.</t>
+    <t xml:space="preserve">Emotional turn: Awe as she becomes real flesh. Holy awe. It becomes real. The Word became flesh and dwelt among us.</t>
   </si>
   <si>
     <t xml:space="preserve">Sculpted (3D). Painterly stylized 3D animation: soft sculpted forms with warm hand-painted textures and real depth and space, like a living storybook in three dimensions, not yet real flesh. Sense: A real breath; the sound of a real heartbeat.</t>
@@ -1121,7 +1127,7 @@
     <t xml:space="preserve">Oil-lamp key light low and warm on hands and bread, soft fill from the fire, deep warm shadows</t>
   </si>
   <si>
-    <t xml:space="preserve">Intimacy. He is with us. Being at home with Him.</t>
+    <t xml:space="preserve">Emotional turn: The warmth of being at home with Him. Intimacy. He is with us. Being at home with Him.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: Warm bread torn open; lamplight; quiet laughter.</t>
@@ -1149,19 +1155,19 @@
     <t xml:space="preserve">Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves; Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane</t>
   </si>
   <si>
-    <t xml:space="preserve">Rosa sits by Samuel's bed and reads to him from a worn Hebrew Bible; glowing letters lift gently from the page and drift into his mind; his tired face softens and he closes his eyes in peace.</t>
+    <t xml:space="preserve">Rosa sits by Samuel's bed and reads to him from a worn Hebrew Bible; glowing letters lift from the page like drops of water and sink into his mind; a tear runs down into his white beard, he reaches out a trembling hand and grips Rosa's, and his lips shape a silent thank you.</t>
   </si>
   <si>
     <t xml:space="preserve">Samuel's small real apartment at night, a lamp, the soup on a tray.</t>
   </si>
   <si>
-    <t xml:space="preserve">Drifts slowly from the open page up to Samuel's face, following the letters. Ends on: Close on Samuel's peaceful face, the light settled within him, Rosa's hand on the page.</t>
+    <t xml:space="preserve">Drifts slowly from the open page up to Samuel's face, following the letters. Ends on: Close on Samuel's tear and his trembling hand holding Rosa's on the page.</t>
   </si>
   <si>
     <t xml:space="preserve">One bedside lamp, warm and low; tiny gold letters rising off the page as small moving lights</t>
   </si>
   <si>
-    <t xml:space="preserve">Comfort; the lonely are visited. His Word bringing life into an old heart.</t>
+    <t xml:space="preserve">Emotional turn: Samuel's tear, his trembling hand, a silent thank you. Comfort; the lonely old man is loved. His Word bringing life into an old heart.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: Pages turning; a soft reading voice; the lamp's warmth.</t>
@@ -1170,7 +1176,7 @@
     <t xml:space="preserve">No caption text; the letters are tiny drifting light; Samuel is frail but not near death or in pain. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. Samuel's small real apartment at night, a lamp, the soup on a tray. Rosa sits by Samuel's bed and reads to him from a worn Hebrew Bible; glowing letters lift gently from the page and drift into his mind; his tired face softens and he closes his eyes in peace. The camera drifts slowly from the open page up to Samuel's face, following the letters. The color stays warm gold, and any light grows slowly from nothing, never flashing. 85mm lens. The shot ends: close on Samuel's peaceful face, the light settled within him, Rosa's hand on the page.
+    <t xml:space="preserve">Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. Samuel's small real apartment at night, a lamp, the soup on a tray. Rosa sits by Samuel's bed and reads to him from a worn Hebrew Bible; glowing letters lift from the page like drops of water and sink into his mind; a tear runs down into his white beard, he reaches out a trembling hand and grips Rosa's, and his lips shape a silent thank you. The camera drifts slowly from the open page up to Samuel's face, following the letters. The color stays warm gold, and any light grows slowly from nothing, never flashing. 85mm lens. The shot ends: close on Samuel's tear and his trembling hand holding Rosa's on the page.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -1201,7 +1207,7 @@
     <t xml:space="preserve">Strong golden sunrise through the window as key light, soft bounce off the walls onto their faces</t>
   </si>
   <si>
-    <t xml:space="preserve">Rising joy. In His presence, you will rise.</t>
+    <t xml:space="preserve">Emotional turn: Three people laughing at the sunlit window. Rising joy. In His presence, you will rise.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: A window opening; morning birds; a cane tapping the floor.</t>
@@ -1238,7 +1244,7 @@
     <t xml:space="preserve">Low golden evening sun backlighting the vine leaves and grapes, warm rim on the family</t>
   </si>
   <si>
-    <t xml:space="preserve">Delight in the fruit of labor. Hard work tastes sweet.</t>
+    <t xml:space="preserve">Emotional turn: A child's grin, the sweetness of the fruit. Delight in the fruit of labor. Hard work tastes sweet.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: Grapes bursting; laughter across the rows.</t>
@@ -1275,7 +1281,7 @@
     <t xml:space="preserve">Warm string lights overhead and late dusk sky; candles on the table; Yeshua lit warmly at the head</t>
   </si>
   <si>
-    <t xml:space="preserve">Celebration; one family of many. The vine's fruit gathered together.</t>
+    <t xml:space="preserve">Emotional turn: A feast of neighbors laughing. Celebration; one family of many. The vine's fruit gathered together.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: Plates clinking; music; many languages laughing.</t>
@@ -1303,19 +1309,19 @@
     <t xml:space="preserve">Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan; Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves; Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat; Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds; Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane; everyone at the long table</t>
   </si>
   <si>
-    <t xml:space="preserve">Everyone at the table joins hands to give thanks; a thread of soft gold light runs from hand to hand down the whole table like a vine.</t>
+    <t xml:space="preserve">Everyone at the table joins hands to give thanks; light flows like warm water from hand to hand down the whole table, and as it reaches each person their face opens: a laugh, a tear, a squeeze of a neighbor's hand.</t>
   </si>
   <si>
     <t xml:space="preserve">The same long table at dusk.</t>
   </si>
   <si>
-    <t xml:space="preserve">Glides along the joined hands in one unbroken move, slowed down. Ends on: Wide on the whole table joined hand to hand, glowing softly.</t>
+    <t xml:space="preserve">Glides along the joined hands in one unbroken move, slowed down. Ends on: Wide on the whole table joined hand to hand, faces glowing and moved.</t>
   </si>
   <si>
     <t xml:space="preserve">Dusk blue sky with warm candle and string-light pools; a soft gold thread of light along the hands</t>
   </si>
   <si>
-    <t xml:space="preserve">Union; one body. Many branches, one vine.</t>
+    <t xml:space="preserve">Emotional turn: Each face opening as the light passes. Union; one body. Many branches, one vine.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: A hush falling over a crowd; hands warm in hands.</t>
@@ -1324,7 +1330,7 @@
     <t xml:space="preserve">The light is a gentle glow, never a laser line or electric spark. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. The same long table at dusk. Everyone at the table joins hands to give thanks; a thread of soft gold light runs from hand to hand down the whole table like a vine. The camera glides along the joined hands in one unbroken move, slowed down. The color stays warm gold, and any light grows slowly from nothing, never flashing. 35mm lens. The shot ends: wide on the whole table joined hand to hand, glowing softly.
+    <t xml:space="preserve">Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. The same long table at dusk. Everyone at the table joins hands to give thanks; light flows like warm water from hand to hand down the whole table, and as it reaches each person their face opens: a laugh, a tear, a squeeze of a neighbor's hand. The camera glides along the joined hands in one unbroken move, slowed down. The color stays warm gold, and any light grows slowly from nothing, never flashing. 35mm lens. The shot ends: wide on the whole table joined hand to hand, faces glowing and moved.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -1340,19 +1346,19 @@
     <t xml:space="preserve">Empty Hands</t>
   </si>
   <si>
-    <t xml:space="preserve">Eli sets his phone face down on the ledge, opens his empty hands, and lifts his face to the sunrise; light gathers in his palms and grows within him.</t>
+    <t xml:space="preserve">Eli sets his phone face down on the ledge, opens his empty hands and lifts his face to the sunrise; light wells up and pools in his palms until it spills over his fingers; he laughs through tears, free.</t>
   </si>
   <si>
     <t xml:space="preserve">A real rooftop at dawn above the city.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pushes in slowly from his open hands to his face. Ends on: Close on Eli's glowing open hands, his peaceful face beyond.</t>
+    <t xml:space="preserve">Pushes in slowly from his open hands to his face. Ends on: Close on Eli's overflowing palms and his laughing, tear-streaked face beyond.</t>
   </si>
   <si>
     <t xml:space="preserve">Clean golden sunrise, low and frontal from the side; light gathering in his palms</t>
   </si>
   <si>
-    <t xml:space="preserve">Surrender. Letting go of the performance for something real.</t>
+    <t xml:space="preserve">Emotional turn: Eli laughs through tears, free. Surrender. Letting go of the performance for something real.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: City waking below; wind on a rooftop.</t>
@@ -1361,7 +1367,7 @@
     <t xml:space="preserve">He does not throw or smash the phone; no lens flare burst. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. A real rooftop at dawn above the city. Eli sets his phone face down on the ledge, opens his empty hands, and lifts his face to the sunrise; light gathers in his palms and grows within him. The camera pushes in slowly from his open hands to his face. The color stays warm gold, and any light grows slowly from nothing, never flashing. 85mm lens, shallow depth of field. The shot ends: close on Eli's glowing open hands, his peaceful face beyond.
+    <t xml:space="preserve">Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. A real rooftop at dawn above the city. Eli sets his phone face down on the ledge, opens his empty hands and lifts his face to the sunrise; light wells up and pools in his palms until it spills over his fingers; he laughs through tears, free. The camera pushes in slowly from his open hands to his face. The color stays warm gold, and any light grows slowly from nothing, never flashing. 85mm lens, shallow depth of field. The shot ends: close on Eli's overflowing palms and his laughing, tear-streaked face beyond.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -1392,7 +1398,7 @@
     <t xml:space="preserve">Cool silver moonlight through olive leaves; a soft warm light on Yeshua only</t>
   </si>
   <si>
-    <t xml:space="preserve">Anguish and surrender. Not my will but Yours.</t>
+    <t xml:space="preserve">Emotional turn: Anguish and surrender in prayer. Anguish and surrender. Not my will but Yours.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: Night crickets; olive leaves in a faint breeze; his breath.</t>
@@ -1429,7 +1435,7 @@
     <t xml:space="preserve">Cold blue night through rainy glass; one warm golden glow outside the window falling across his face</t>
   </si>
   <si>
-    <t xml:space="preserve">Despair, and a crack of hope. The end of himself, and the first turning.</t>
+    <t xml:space="preserve">Emotional turn: Despair, and the first lifted head. Despair, and a crack of hope. The end of himself, and the first turning.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: Rain on glass; a single shaking breath.</t>
@@ -1469,7 +1475,7 @@
     <t xml:space="preserve">The warm window light now inside the room, spreading around them like lamplight</t>
   </si>
   <si>
-    <t xml:space="preserve">Being found. He was never alone, not for one moment.</t>
+    <t xml:space="preserve">Emotional turn: David breaks down, found. Being found. He was never alone, not for one moment.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: Weeping that loosens; a hand's warmth through a jacket.</t>
@@ -1509,7 +1515,7 @@
     <t xml:space="preserve">Harsh dusty midday sun, high and hard, warmed toward gold; no stylized drama</t>
   </si>
   <si>
-    <t xml:space="preserve">Sacrificial love; quiet strength. Love that carries what is not its own.</t>
+    <t xml:space="preserve">Emotional turn: Quiet, steady love carrying the beam. Sacrificial love; quiet strength. Love that carries what is not its own.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: Wood scraping stone; a crowd's murmur; his breathing.</t>
@@ -1537,19 +1543,19 @@
     <t xml:space="preserve">Rosa, Tomas, Eli, Samuel and David, and the crossbeam passing through the crowd</t>
   </si>
   <si>
-    <t xml:space="preserve">From Rosa's tired shoulders, Tomas's load, Eli's empty performance, Samuel's sickness and David's shame, dark threads like ash lift away and drift toward the crossbeam passing through the crowd; each person straightens, lighter.</t>
+    <t xml:space="preserve">From Rosa's tired shoulders, Tomas's load, Eli's empty performance, Samuel's sickness and David's shame, dark threads like ash lift away and drift toward the crossbeam passing through the crowd; one after another they straighten, breathe in deeply, and their faces break with relief and grateful tears.</t>
   </si>
   <si>
     <t xml:space="preserve">Intercut in one continuous move: the apartment building and the Jerusalem street become one space.</t>
   </si>
   <si>
-    <t xml:space="preserve">Flows from one person to the next, following the drifting threads toward the beam. Ends on: Medium on the crossbeam passing, the drifting threads sinking into the wood.</t>
+    <t xml:space="preserve">Flows from one person to the next, following the drifting threads toward the beam. Ends on: Medium on the crossbeam passing, the drifting threads sinking into the wood, relieved faces behind it.</t>
   </si>
   <si>
     <t xml:space="preserve">Dusty warm daylight; the dark ash-threads catching light as they drift toward the beam</t>
   </si>
   <si>
-    <t xml:space="preserve">Release; burdens lifted. He takes what we could not carry.</t>
+    <t xml:space="preserve">Emotional turn: Burdens lifted: relief and grateful tears. Release; burdens lifted. He takes what we could not carry.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: A deep exhale from many people at once.</t>
@@ -1558,7 +1564,7 @@
     <t xml:space="preserve">No black smoke horror; threads drift gently like ash in warm air; no blood. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. David, a gaunt man in his thirties with unkempt dark hair, stubble and a worn leather jacket. Intercut in one continuous move: the apartment building and the Jerusalem street become one space. From Rosa's tired shoulders, Tomas's load, Eli's empty performance, Samuel's sickness and David's shame, dark threads like ash lift away and drift toward the crossbeam passing through the crowd; each person straightens, lighter. The camera flows from one person to the next, following the drifting threads toward the beam. The color stays warm gold, and any light grows slowly from nothing, never flashing. 50mm lens. The shot ends: medium on the crossbeam passing, the drifting threads sinking into the wood.
+    <t xml:space="preserve">Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. David, a gaunt man in his thirties with unkempt dark hair, stubble and a worn leather jacket. Intercut in one continuous move: the apartment building and the Jerusalem street become one space. From Rosa's tired shoulders, Tomas's load, Eli's empty performance, Samuel's sickness and David's shame, dark threads like ash lift away and drift toward the crossbeam passing through the crowd; one after another they straighten, breathe in deeply, and their faces break with relief and grateful tears. The camera flows from one person to the next, following the drifting threads toward the beam. The color stays warm gold, and any light grows slowly from nothing, never flashing. 50mm lens. The shot ends: medium on the crossbeam passing, the drifting threads sinking into the wood, relieved faces behind it.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -1589,7 +1595,7 @@
     <t xml:space="preserve">Heavy dark sky; gold rays breaking slowly through cloud behind the cross as the only bright source</t>
   </si>
   <si>
-    <t xml:space="preserve">Love poured out. Everything given, nothing held back.</t>
+    <t xml:space="preserve">Emotional turn: Everything given. Love poured out. Everything given, nothing held back.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: Wind on the hill; then stillness.</t>
@@ -1629,7 +1635,7 @@
     <t xml:space="preserve">Warm dusk afterglow on their faces; tears catching the light</t>
   </si>
   <si>
-    <t xml:space="preserve">Gratitude beyond words. Thank You.</t>
+    <t xml:space="preserve">Emotional turn: Joy through tears on the rooftop. Gratitude beyond words. Thank You.</t>
   </si>
   <si>
     <t xml:space="preserve">Flesh (real). Photoreal live-action cinematography: real people with natural, textured skin and pores, real breath and real light. Sense: Quiet crying that turns into a laugh.</t>
@@ -1654,7 +1660,7 @@
     <t xml:space="preserve">The empty rock tomb and a swarm of glowing Hebrew letters rising from it</t>
   </si>
   <si>
-    <t xml:space="preserve">Warm light pours out of the empty tomb, and a swarm of glowing Hebrew letters rises from inside like stars set free, streaming out over the city.</t>
+    <t xml:space="preserve">Warm light pours out of the empty tomb like a spring bursting open, running out across the stone threshold like water, and a swarm of glowing Hebrew letters rises from it like stars set free, streaming out over the city.</t>
   </si>
   <si>
     <t xml:space="preserve">A garden at dawn, a great round stone rolled away from a rock tomb.</t>
@@ -1666,7 +1672,7 @@
     <t xml:space="preserve">Dawn garden light; intense warm light pouring out of the tomb doorway as the main source</t>
   </si>
   <si>
-    <t xml:space="preserve">Victory. Life wins. He is risen; the Word lives.</t>
+    <t xml:space="preserve">Emotional turn: Victory: the spring bursts open. Victory. Life wins. He is risen; the Word lives.</t>
   </si>
   <si>
     <t xml:space="preserve">Glory. Photoreal people transfigured into light: their bodies glowing from within, the edges of their forms dissolving into drifting points of golden light and tiny Hebrew letters. Sense: Morning birds; a rush like wind.</t>
@@ -1675,7 +1681,7 @@
     <t xml:space="preserve">No figure of Jesus inside; no flash; the letters rise slowly. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Photoreal people transfigured into light: their bodies glowing from within, the edges of their forms dissolving into drifting points of golden light and tiny Hebrew letters. A garden at dawn, a great round stone rolled away from a rock tomb. Warm light pours out of the empty tomb, and a swarm of glowing Hebrew letters rises from inside like stars set free, streaming out over the city. The camera pushes in toward the open tomb from ground level, then tilts up with the rising letters. The color stays warm gold, and any light grows slowly from nothing, never flashing. 35mm lens. The shot ends: medium-low on the tomb doorway, letters of light streaming upward.
+    <t xml:space="preserve">Photoreal people transfigured into light: their bodies glowing from within, the edges of their forms dissolving into drifting points of golden light and tiny Hebrew letters. A garden at dawn, a great round stone rolled away from a rock tomb. Warm light pours out of the empty tomb like a spring bursting open, running out across the stone threshold like water, and a swarm of glowing Hebrew letters rises from it like stars set free, streaming out over the city. The camera pushes in toward the open tomb from ground level, then tilts up with the rising letters. The color stays warm gold, and any light grows slowly from nothing, never flashing. 35mm lens. The shot ends: medium-low on the tomb doorway, letters of light streaming upward.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -1694,19 +1700,19 @@
     <t xml:space="preserve">David, a gaunt man in his thirties with unkempt dark hair, stubble and a worn leather jacket; Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane</t>
   </si>
   <si>
-    <t xml:space="preserve">David walks up the street toward home with his head down; Samuel, healed, drops his cane and runs to him, robe flying, and throws his arms around his son; both begin to shine from within.</t>
+    <t xml:space="preserve">David walks up the street toward home with his head down; Samuel, healed, sees him, drops his cane and runs to him, robe flying; David falls into his father's arms sobbing, Samuel laughing and weeping and kissing his head, and light wells up and overflows from both of them like water.</t>
   </si>
   <si>
     <t xml:space="preserve">The street in front of the apartment building at sunrise.</t>
   </si>
   <si>
-    <t xml:space="preserve">Tracks with the running father, right to left, and settles on the embrace. Ends on: Medium on father and son in a tight, glowing embrace.</t>
+    <t xml:space="preserve">Tracks with the running father, right to left, and settles on the embrace. Ends on: Medium on father and son in a tight embrace, crying and laughing, light spilling from them.</t>
   </si>
   <si>
     <t xml:space="preserve">Low gold sunrise down the street, behind David; both begin to glow from within</t>
   </si>
   <si>
-    <t xml:space="preserve">Homecoming; the dead come alive. The son who was lost is found.</t>
+    <t xml:space="preserve">Emotional turn: The father runs; the son falls into his arms. Homecoming; the dead come alive. The son who was lost is found.</t>
   </si>
   <si>
     <t xml:space="preserve">Glory. Photoreal people transfigured into light: their bodies glowing from within, the edges of their forms dissolving into drifting points of golden light and tiny Hebrew letters. Sense: A cane clattering on pavement; a father's cry; sobbing laughter.</t>
@@ -1715,7 +1721,7 @@
     <t xml:space="preserve">Not slow-motion cliché throughout; no lens flare; faces joyful. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Photoreal people transfigured into light: their bodies glowing from within, the edges of their forms dissolving into drifting points of golden light and tiny Hebrew letters. David, a gaunt man in his thirties with unkempt dark hair, stubble and a worn leather jacket. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. The street in front of the apartment building at sunrise. David walks up the street toward home with his head down; Samuel, healed, drops his cane and runs to him, robe flying, and throws his arms around his son; both begin to shine from within. The camera tracks with the running father, right to left, and settles on the embrace. The color stays warm gold, and any light grows slowly from nothing, never flashing. 50mm lens. The shot ends: medium on father and son in a tight, glowing embrace.
+    <t xml:space="preserve">Photoreal people transfigured into light: their bodies glowing from within, the edges of their forms dissolving into drifting points of golden light and tiny Hebrew letters. David, a gaunt man in his thirties with unkempt dark hair, stubble and a worn leather jacket. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. The street in front of the apartment building at sunrise. David walks up the street toward home with his head down; Samuel, healed, sees him, drops his cane and runs to him, robe flying; David falls into his father's arms sobbing, Samuel laughing and weeping and kissing his head, and light wells up and overflows from both of them like water. The camera tracks with the running father, right to left, and settles on the embrace. The color stays warm gold, and any light grows slowly from nothing, never flashing. 50mm lens. The shot ends: medium on father and son in a tight embrace, crying and laughing, light spilling from them.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -1734,7 +1740,7 @@
     <t xml:space="preserve">Yeshua shining with a gentle golden glory, small in the frame; Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan; Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves; Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat; Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds; Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane; David, a gaunt man in his thirties with unkempt dark hair, stubble and a worn leather jacket; a countless crowd of every nation and age</t>
   </si>
   <si>
-    <t xml:space="preserve">Ana, Rosa, Tomas, Eli, Samuel and David stand among a countless crowd, all transfigured into light, turned toward Yeshua shining at the center; their many lights flow together like one long bridal veil across the hill.</t>
+    <t xml:space="preserve">Ana, Rosa, Tomas, Eli, Samuel and David stand among a countless crowd of every nation, faces wet with joy, embracing, turned toward Yeshua shining at the center; streams of light overflow from every person, run downhill together and join into one shining river, flowing out like a bridal veil across the hill.</t>
   </si>
   <si>
     <t xml:space="preserve">A vast vineyard hillside at sunrise filled with people of every nation and every age.</t>
@@ -1746,7 +1752,7 @@
     <t xml:space="preserve">Wide golden sunrise over the hillside; every person a soft source of their own light; Yeshua brightest, gentle</t>
   </si>
   <si>
-    <t xml:space="preserve">Glory; all made one. The Bride, gathered to Him.</t>
+    <t xml:space="preserve">Emotional turn: Every face wet with joy, one river. Glory; all made one. The Bride, gathered to Him.</t>
   </si>
   <si>
     <t xml:space="preserve">Glory. Photoreal people transfigured into light: their bodies glowing from within, the edges of their forms dissolving into drifting points of golden light and tiny Hebrew letters. Sense: A great hush, then joy like many waters.</t>
@@ -1755,7 +1761,7 @@
     <t xml:space="preserve">Not a stadium concert crowd; no raised-hands stock-photo look; Yeshua small and radiant, never singing. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Photoreal people transfigured into light: their bodies glowing from within, the edges of their forms dissolving into drifting points of golden light and tiny Hebrew letters. Yeshua, a first-century Galilean Jewish man in his early thirties, six feet tall and noticeably taller than those around him, lean and weathered with sun-tanned olive skin, calloused hands, dark brown hair to the nape of his neck, a full dark beard and dark brown eyes, wears a plain undyed cream tunic belted at the waist and a large cream rectangular mantle with dark stripes and knotted tassels at its four corners, with leather sandals. He shines with a gentle golden glory from within, steady and calm, never a flash. Seen from a distance, he stays small in the frame and is never turned squarely toward the camera. He never sings or mouths words. Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. David, a gaunt man in his thirties with unkempt dark hair, stubble and a worn leather jacket. A vast vineyard hillside at sunrise filled with people of every nation and every age. Ana, Rosa, Tomas, Eli, Samuel and David stand among a countless crowd, all transfigured into light, turned toward Yeshua shining at the center; their many lights flow together like one long bridal veil across the hill. The camera pulls back and rises in a slow drone move from their faces to the whole gathering. The color stays warm gold, and any light grows slowly from nothing, never flashing. Wide lens, deep focus. The shot ends: high and wide, the shining crowd one whole around Yeshua.
+    <t xml:space="preserve">Photoreal people transfigured into light: their bodies glowing from within, the edges of their forms dissolving into drifting points of golden light and tiny Hebrew letters. Yeshua, a first-century Galilean Jewish man in his early thirties, six feet tall and noticeably taller than those around him, lean and weathered with sun-tanned olive skin, calloused hands, dark brown hair to the nape of his neck, a full dark beard and dark brown eyes, wears a plain undyed cream tunic belted at the waist and a large cream rectangular mantle with dark stripes and knotted tassels at its four corners, with leather sandals. He shines with a gentle golden glory from within, steady and calm, never a flash. Seen from a distance, he stays small in the frame and is never turned squarely toward the camera. He never sings or mouths words. Ana, a girl of eight with dark curly hair in two braids and a yellow cardigan. Rosa, a Latina woman in her mid-forties with dark hair tied back, tired kind eyes, a navy cleaning-company uniform and yellow rubber gloves. Tomas, a broad-shouldered construction worker in his forties with a short greying beard, an orange safety vest and a scuffed white hard hat. Eli, a Black teenage boy of seventeen with short twists, a grey hooded sweatshirt and white earbuds. Samuel, a frail Jewish man in his eighties with a white beard, a knitted cardigan and a wooden cane. David, a gaunt man in his thirties with unkempt dark hair, stubble and a worn leather jacket. A vast vineyard hillside at sunrise filled with people of every nation and every age. Ana, Rosa, Tomas, Eli, Samuel and David stand among a countless crowd of every nation, faces wet with joy, embracing, turned toward Yeshua shining at the center; streams of light overflow from every person, run downhill together and join into one shining river, flowing out like a bridal veil across the hill. The camera pulls back and rises in a slow drone move from their faces to the whole gathering. The color stays warm gold, and any light grows slowly from nothing, never flashing. Wide lens, deep focus. The shot ends: high and wide, the shining crowd one whole around Yeshua.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -1774,19 +1780,19 @@
     <t xml:space="preserve">Countless small lights of people joined into one vine of light across the earth</t>
   </si>
   <si>
-    <t xml:space="preserve">Countless small golden lights of people across cities, villages and fields join by glowing threads of Hebrew letters into one great living vine of light that branches across the whole earth, the same vine from the first frame, now made of people.</t>
+    <t xml:space="preserve">Countless small golden springs of light, people across cities, villages and fields, flow together into one great river of living light that branches across the whole earth like a vine, the same vine from the first frames, now made of people.</t>
   </si>
   <si>
     <t xml:space="preserve">High above the earth at dawn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Rises slowly higher in a smooth, floating move. Ends on: Very high and wide, the vine of light spread across the earth, fading to warm gold-white.</t>
+    <t xml:space="preserve">Rises slowly higher in a smooth, floating move. Ends on: Very high and wide, the river-vine of light spread across the earth, fading to warm gold-white for the Dazadi Music credit.</t>
   </si>
   <si>
     <t xml:space="preserve">Dawn over the land; the vine of people-light glowing gold, fading toward warm gold-white</t>
   </si>
   <si>
-    <t xml:space="preserve">Eternity; peace. We are His and He is ours; the circle is complete.</t>
+    <t xml:space="preserve">Emotional turn: Peace: the circle complete. Eternity; peace. We are His and He is ours; the circle is complete.</t>
   </si>
   <si>
     <t xml:space="preserve">Glory. Photoreal people transfigured into light: their bodies glowing from within, the edges of their forms dissolving into drifting points of golden light and tiny Hebrew letters. Sense: The low hum from the first frame returning, warm and full.</t>
@@ -1795,7 +1801,7 @@
     <t xml:space="preserve">No planet-from-space cliché; no text; fade softly toward warm golden white for the credit. Standing: no English words or captions; no pink or neon; no vignette or color grade; no plastic skin; no blood; no jarring cuts; light never flashes; Yeshua never sings, never full face-on, kneels only in prayer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Photoreal people transfigured into light: their bodies glowing from within, the edges of their forms dissolving into drifting points of golden light and tiny Hebrew letters. High above the earth at dawn. Countless small golden lights of people across cities, villages and fields join by glowing threads of Hebrew letters into one great living vine of light that branches across the whole earth, the same vine from the first frame, now made of people. The camera rises slowly higher in a smooth, floating move. The color stays warm gold, and any light grows slowly from nothing, never flashing. Wide lens, deep focus. The shot ends: very high and wide, the vine of light spread across the earth, fading to warm gold-white.
+    <t xml:space="preserve">Photoreal people transfigured into light: their bodies glowing from within, the edges of their forms dissolving into drifting points of golden light and tiny Hebrew letters. High above the earth at dawn. Countless small golden springs of light, people across cities, villages and fields, flow together into one great river of living light that branches across the whole earth like a vine, the same vine from the first frames, now made of people. The camera rises slowly higher in a smooth, floating move. The color stays warm gold, and any light grows slowly from nothing, never flashing. Wide lens, deep focus. The shot ends: very high and wide, the river-vine of light spread across the earth, fading to warm gold-white for the Dazadi Music credit.
 AVOID: English words, captions, titles or lyric text (Hebrew letters appear only as drifting light, never as a caption), black bars, white edge lines, collage or grid, vignette, color grade, pink tint or neon light (keep warm gold), plastic or overly smooth skin, film grain, jarring cuts, blood, halos or light flashes; Yeshua never sings or mouths words; Yeshua's face never shown full and head-on; he kneels only when praying.</t>
   </si>
   <si>
@@ -2409,7 +2415,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -2429,7 +2435,7 @@
       <c r="A3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2439,28 +2445,41 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>4</v>
-      </c>
+      <c r="A6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -2501,2262 +2520,2262 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C2" s="5" t="n">
         <v>7</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="P2" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C3" s="5" t="n">
         <v>6</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>7</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>6</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="P5" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>6</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>6</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O7" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>7</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O8" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>6</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O9" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P9" s="7" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>7</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O10" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P10" s="7" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C11" s="7" t="n">
         <v>7</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O11" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P11" s="7" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>8</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="M12" s="7" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="N12" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O12" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P12" s="7" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>7</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O13" s="7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="P13" s="7" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C14" s="7" t="n">
         <v>7</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="N14" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O14" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P14" s="7" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C15" s="7" t="n">
         <v>7</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="N15" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O15" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P15" s="7" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C16" s="7" t="n">
         <v>7</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="N16" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O16" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P16" s="7" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C17" s="9" t="n">
         <v>6</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F17" s="9"/>
       <c r="G17" s="9" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="I17" s="9" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="L17" s="9" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M17" s="9" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O17" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C18" s="9" t="n">
         <v>7</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="L18" s="9" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="M18" s="9" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="N18" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O18" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P18" s="9" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C19" s="9" t="n">
         <v>7</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="M19" s="9" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P19" s="9" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C20" s="9" t="n">
         <v>7</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="L20" s="9" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="M20" s="9" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="N20" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O20" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P20" s="9" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C21" s="9" t="n">
         <v>6</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="M21" s="9" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C22" s="9" t="n">
         <v>7</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="L22" s="9" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="M22" s="9" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="N22" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O22" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P22" s="9" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C23" s="9" t="n">
         <v>6</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="L23" s="9" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="M23" s="9" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O23" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C24" s="9" t="n">
         <v>7</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="J24" s="9" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="K24" s="9" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="L24" s="9" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="M24" s="9" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="N24" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O24" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P24" s="9" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C25" s="9" t="n">
         <v>8</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="L25" s="9" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="M25" s="9" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P25" s="9" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C26" s="9" t="n">
         <v>8</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L26" s="9" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="M26" s="9" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="N26" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O26" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P26" s="9" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C27" s="9" t="n">
         <v>8</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="L27" s="9" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="M27" s="9" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C28" s="11" t="n">
         <v>8</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="K28" s="11" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="L28" s="11" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="M28" s="11" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="N28" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O28" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P28" s="11" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="C29" s="11" t="n">
         <v>7</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="K29" s="11" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="L29" s="11" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="M29" s="11" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="N29" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O29" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P29" s="11" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="C30" s="11" t="n">
         <v>8</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="K30" s="11" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="L30" s="11" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="M30" s="11" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="N30" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O30" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P30" s="11" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C31" s="11" t="n">
         <v>6</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="K31" s="11" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="L31" s="11" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="M31" s="11" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="N31" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O31" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P31" s="11" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C32" s="11" t="n">
         <v>6</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="K32" s="11" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="L32" s="11" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="M32" s="11" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="N32" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O32" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P32" s="11" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="C33" s="11" t="n">
         <v>6</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="K33" s="11" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="L33" s="11" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="M33" s="11" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="N33" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O33" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P33" s="11" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="C34" s="11" t="n">
         <v>7</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="H34" s="11" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="K34" s="11" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="L34" s="11" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="M34" s="11" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="N34" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O34" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P34" s="11" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="C35" s="11" t="n">
         <v>7</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="H35" s="11" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="K35" s="11" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="L35" s="11" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="M35" s="11" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="N35" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O35" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P35" s="11" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C36" s="11" t="n">
         <v>6</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="H36" s="11" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="K36" s="11" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="L36" s="11" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="M36" s="11" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="N36" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O36" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P36" s="11" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="C37" s="11" t="n">
         <v>7</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="H37" s="11" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="K37" s="11" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="L37" s="11" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="M37" s="11" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="N37" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O37" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P37" s="11" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="C38" s="11" t="n">
         <v>6</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="H38" s="11" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="K38" s="11" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="L38" s="11" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="M38" s="11" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="N38" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O38" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P38" s="11" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="C39" s="11" t="n">
         <v>6</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="H39" s="11" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="K39" s="11" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="L39" s="11" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="M39" s="11" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="N39" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O39" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P39" s="11" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="C40" s="11" t="n">
         <v>6</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="H40" s="11" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="K40" s="11" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="L40" s="11" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="M40" s="11" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="N40" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O40" s="11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="P40" s="11" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="C41" s="11" t="n">
         <v>6</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="G41" s="11" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="H41" s="11" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="K41" s="11" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="L41" s="11" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="M41" s="11" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="N41" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O41" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P41" s="11" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>6</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="F42" s="13" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="G42" s="13" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="H42" s="13" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="I42" s="13" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="J42" s="13" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="K42" s="13" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="L42" s="13" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="M42" s="13" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="N42" s="13" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O42" s="13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="P42" s="13" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="12" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>7</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="F43" s="13" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="G43" s="13" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="H43" s="13" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="I43" s="13" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="J43" s="13" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="K43" s="13" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L43" s="13" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="M43" s="13" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="N43" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O43" s="13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P43" s="13" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>7</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="F44" s="13" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="G44" s="13" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H44" s="13" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="I44" s="13" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="J44" s="13" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="K44" s="13" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="L44" s="13" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="M44" s="13" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="N44" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O44" s="13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="P44" s="13" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="210" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>6</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="F45" s="13" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="G45" s="13" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="H45" s="13" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="I45" s="13" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="J45" s="13" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="K45" s="13" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="L45" s="13" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="M45" s="13" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="N45" s="13" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O45" s="13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="P45" s="13" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="14" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="C46" s="14" t="n">
         <f aca="false">SUM(C2:C45)</f>
         <v>296</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
   </sheetData>
@@ -4786,90 +4805,90 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
     </row>
   </sheetData>

</xml_diff>